<commit_message>
feat: generalize construction cost estimates for multi-country use
</commit_message>
<xml_diff>
--- a/outputs/koica-construction-distribution/KOICA_건축사업_사례라이브러리_2016-2025.xlsx
+++ b/outputs/koica-construction-distribution/KOICA_건축사업_사례라이브러리_2016-2025.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Ra41c074edfd641e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검토사례" sheetId="2" r:id="R4e858807eaa04a6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="표본현황" sheetId="3" r:id="R7b7fe770bf7d4910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터사전" sheetId="4" r:id="R970743d119a9493d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL 예시" sheetId="5" r:id="R17c58fce45f14a2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Rda15b7a2987a48aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검토사례" sheetId="2" r:id="Ra2c5b37405684bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="표본현황" sheetId="3" r:id="R8ee6e73d65c6424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="국가지수현황" sheetId="4" r:id="R03fae5b2d6a645f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터사전" sheetId="5" r:id="R5c42feaf85534f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL 예시" sheetId="6" r:id="Rad8ded3cd6ef4ae5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,10 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0.000"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="202" formatCode="&quot;$&quot;#,##0"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0"/>
+    <x:numFmt numFmtId="204" formatCode="yyyy-mm-dd hh:mm"/>
   </x:numFmts>
   <x:fonts count="8">
     <x:font>
@@ -141,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -243,11 +246,29 @@
     <x:xf numFmtId="202" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="3">
     <x:dxf>
       <x:font>
         <x:color rgb="FF9C0006"/>
@@ -268,13 +289,23 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{08B1EED1-66B5-4936-9680-4A547F515FDE}"/>
+  <xltc:person displayName="User" id="{C51560CE-245F-46B0-A622-F8E49E70857B}"/>
 </xltc:personList>
 </file>
 
@@ -329,7 +360,35 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DataDictionary" displayName="DataDictionary" ref="A2:C14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CountryPriceIndexStatus" displayName="CountryPriceIndexStatus" ref="A2:T30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="20">
+    <x:tableColumn id="1" name="국가"/>
+    <x:tableColumn id="2" name="ISO3"/>
+    <x:tableColumn id="3" name="검토사례수"/>
+    <x:tableColumn id="4" name="공식후보_우선순위"/>
+    <x:tableColumn id="5" name="공식후보_지수명"/>
+    <x:tableColumn id="6" name="공식후보_제공기관"/>
+    <x:tableColumn id="7" name="감사상태"/>
+    <x:tableColumn id="8" name="공식후보_URL"/>
+    <x:tableColumn id="9" name="현재선택_우선순위"/>
+    <x:tableColumn id="10" name="현재선택_지수분류"/>
+    <x:tableColumn id="11" name="현재선택_지수명"/>
+    <x:tableColumn id="12" name="현재선택_제공기관"/>
+    <x:tableColumn id="13" name="주기"/>
+    <x:tableColumn id="14" name="실제관측값수"/>
+    <x:tableColumn id="15" name="최초기간"/>
+    <x:tableColumn id="16" name="최근기간"/>
+    <x:tableColumn id="17" name="최근값상태"/>
+    <x:tableColumn id="18" name="최근조회시각"/>
+    <x:tableColumn id="19" name="현재선택_URL"/>
+    <x:tableColumn id="20" name="자동사용_주의사항"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DataDictionary" displayName="DataDictionary" ref="A2:C18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="테이블·뷰"/>
     <x:tableColumn id="2" name="내용"/>
@@ -339,8 +398,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SqlExamples" displayName="SqlExamples" ref="A2:B7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SqlExamples" displayName="SqlExamples" ref="A2:B9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="목적"/>
     <x:tableColumn id="2" name="SQL"/>
@@ -628,12 +687,26 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="13" t="str">
+        <x:v>국가별 적용 분기</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="90" customHeight="1">
+      <x:c r="A22" s="16" t="str">
+        <x:v>• 동일 국가 사례+공식 건설지수: 범위·기간을 맞춘 뒤 교차검증
+• 동일 국가 사례만 있음: 현지 견적을 주자료로 하고 지수 부재를 명시
+• 동일 국가 사례 없음: 타 국가 사례는 설계·공종 참고에만 사용
+• 수입재 비중 큼: 현지비와 수입비를 통화·공급국별로 분리
+• 기준일까지 지수 미공개: 관측종료일까지만 계산하고 이후는 시나리오</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="13" t="str">
         <x:v>미래 사업 조사 절차</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="66" customHeight="1">
-      <x:c r="A22" s="23" t="str">
-        <x:v>1) SQLite에서 국가·시설·사업유형이 유사한 사례 검색 → 2) A/B등급 원문 확인 → 3) 현지 QS 개략견적·BOQ 및 시공사 견적 2~3개 확보 → 4) 공고일 기준 물가·환율·세금·범위 보정 → 5) 보정 근거와 불확실성을 보고서에 기록</x:v>
+    <x:row r="31" ht="82" customHeight="1">
+      <x:c r="A31" s="23" t="str">
+        <x:v>1) 국가별 템플릿의 사업 입력·비용경계 작성 → 2) SQLite에서 국가·시설·사업유형이 유사한 사례 검색 → 3) A/B등급 원문과 가격단계·세금·범위 확인 → 4) 현지 QS 개략견적·BOQ 및 시공사 견적 2~3개 확보 → 5) 실제 관측 지수의 원래 기간·잠정상태·관측종료일 기록 → 6) 통화·수입재 구성 확인 후 보정 → 7) 복수변수 시나리오와 불확실성 보고</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -645,7 +718,9 @@
     <x:mergeCell ref="A14:H14"/>
     <x:mergeCell ref="A15:H18"/>
     <x:mergeCell ref="A21:H21"/>
-    <x:mergeCell ref="A22:H26"/>
+    <x:mergeCell ref="A22:H27"/>
+    <x:mergeCell ref="A30:H30"/>
+    <x:mergeCell ref="A31:H36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1920,7 +1995,7 @@
         <x:v>공사 입찰 집행한도</x:v>
       </x:c>
       <x:c r="O19" s="36" t="str">
-        <x:v>산업시설 성격</x:v>
+        <x:v>산업시설·지하 1층 포함; 첨부 추정가격 USD 3,446,170과 상세페이지 집행한도 USD 3,534,542가 상이; VAT 제외</x:v>
       </x:c>
       <x:c r="P19" s="33" t="str">
         <x:v>미보정</x:v>
@@ -1944,7 +2019,7 @@
         <x:v>https://nebid.koica.go.kr/oep/lobi/localBidManageDetail.do?P_LOAZ_BID_PBLANC_NO=L2024-00079&amp;P_PBLANC_ODR=1</x:v>
       </x:c>
       <x:c r="W19" s="36" t="str">
-        <x:v>총연면적 4,996.62㎡; 상세페이지 집행한도 USD 3,534,542; 산출단가 USD 707/㎡.</x:v>
+        <x:v>총연면적 4,996.62㎡(지하 1층 포함); 첨부 추정가격 USD 3,446,170(약 USD 690/㎡), 상세페이지 집행한도 USD 3,534,542(약 USD 707/㎡); VAT 제외.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3526,7 +3601,9 @@
       <x:c r="N42" s="36" t="str">
         <x:v>공사 입찰 집행한도</x:v>
       </x:c>
-      <x:c r="O42" s="36" t="str"/>
+      <x:c r="O42" s="36" t="str">
+        <x:v>건물공사와 외부토목·조경·주차·배수 등 포함; VAT 제외</x:v>
+      </x:c>
       <x:c r="P42" s="33" t="str">
         <x:v>미보정</x:v>
       </x:c>
@@ -3549,7 +3626,7 @@
         <x:v>https://nebid.koica.go.kr/oep/lobi/localBidManageDetail.do?P_LOAZ_BID_PBLANC_NO=L2022-00029&amp;P_PBLANC_ODR=1</x:v>
       </x:c>
       <x:c r="W42" s="36" t="str">
-        <x:v>총연면적 5,640.10㎡; 상세페이지 집행한도 USD 3,744,400; 산출단가 USD 664/㎡.</x:v>
+        <x:v>총연면적 5,640.10㎡; 상세페이지 집행한도 USD 3,744,400; 건물·외부공사 포함; VAT 제외; 산출단가 USD 664/㎡.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -4689,7 +4766,9 @@
       <x:c r="N59" s="36" t="str">
         <x:v>공사 입찰 집행한도</x:v>
       </x:c>
-      <x:c r="O59" s="36" t="str"/>
+      <x:c r="O59" s="36" t="str">
+        <x:v>VAT 제외; 외부공사 등 포함범위 재확인</x:v>
+      </x:c>
       <x:c r="P59" s="33" t="str">
         <x:v>미보정</x:v>
       </x:c>
@@ -5335,7 +5414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81382889834f440f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b69f1a8c9724e2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7648,12 +7727,1815 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43cc8fbfa2fb48dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93046aa8c2f34a0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="13" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="46" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="13" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="30" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="13" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="46" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="25" t="str">
+        <x:v>28개국 가격지수 후보·현재 선택·관측상태</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="27" t="str">
+        <x:v>국가</x:v>
+      </x:c>
+      <x:c r="B2" s="27" t="str">
+        <x:v>ISO3</x:v>
+      </x:c>
+      <x:c r="C2" s="27" t="str">
+        <x:v>검토사례수</x:v>
+      </x:c>
+      <x:c r="D2" s="27" t="str">
+        <x:v>공식후보_우선순위</x:v>
+      </x:c>
+      <x:c r="E2" s="27" t="str">
+        <x:v>공식후보_지수명</x:v>
+      </x:c>
+      <x:c r="F2" s="27" t="str">
+        <x:v>공식후보_제공기관</x:v>
+      </x:c>
+      <x:c r="G2" s="27" t="str">
+        <x:v>감사상태</x:v>
+      </x:c>
+      <x:c r="H2" s="27" t="str">
+        <x:v>공식후보_URL</x:v>
+      </x:c>
+      <x:c r="I2" s="27" t="str">
+        <x:v>현재선택_우선순위</x:v>
+      </x:c>
+      <x:c r="J2" s="27" t="str">
+        <x:v>현재선택_지수분류</x:v>
+      </x:c>
+      <x:c r="K2" s="27" t="str">
+        <x:v>현재선택_지수명</x:v>
+      </x:c>
+      <x:c r="L2" s="27" t="str">
+        <x:v>현재선택_제공기관</x:v>
+      </x:c>
+      <x:c r="M2" s="27" t="str">
+        <x:v>주기</x:v>
+      </x:c>
+      <x:c r="N2" s="27" t="str">
+        <x:v>실제관측값수</x:v>
+      </x:c>
+      <x:c r="O2" s="27" t="str">
+        <x:v>최초기간</x:v>
+      </x:c>
+      <x:c r="P2" s="27" t="str">
+        <x:v>최근기간</x:v>
+      </x:c>
+      <x:c r="Q2" s="27" t="str">
+        <x:v>최근값상태</x:v>
+      </x:c>
+      <x:c r="R2" s="27" t="str">
+        <x:v>최근조회시각</x:v>
+      </x:c>
+      <x:c r="S2" s="27" t="str">
+        <x:v>현재선택_URL</x:v>
+      </x:c>
+      <x:c r="T2" s="27" t="str">
+        <x:v>자동사용_주의사항</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="32" t="str">
+        <x:v>Bangladesh</x:v>
+      </x:c>
+      <x:c r="B3" s="32" t="str">
+        <x:v>BGD</x:v>
+      </x:c>
+      <x:c r="C3" s="32" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D3" s="32" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E3" s="35" t="str">
+        <x:v>Building Materials Price Index (BMPI)</x:v>
+      </x:c>
+      <x:c r="F3" s="35" t="str">
+        <x:v>Bangladesh Bureau of Statistics</x:v>
+      </x:c>
+      <x:c r="G3" s="35" t="str">
+        <x:v>공식 후보 확인·시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H3" s="35" t="str">
+        <x:v>https://bbs.gov.bd/site/page/29b379ff-7bac-41d9-b321-e41929bab4a1</x:v>
+      </x:c>
+      <x:c r="I3" s="32" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J3" s="35" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K3" s="35" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L3" s="35" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M3" s="32" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N3" s="47" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O3" s="32" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P3" s="32" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q3" s="35" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R3" s="50" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S3" s="35" t="str">
+        <x:v>https://api.worldbank.org/v2/country/BGD/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T3" s="35" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="33" t="str">
+        <x:v>Bolivia</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>BOL</x:v>
+      </x:c>
+      <x:c r="C4" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D4" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="36" t="str">
+        <x:v>Índice de Costo de la Construcción (ICC)</x:v>
+      </x:c>
+      <x:c r="F4" s="36" t="str">
+        <x:v>Instituto Nacional de Estadística</x:v>
+      </x:c>
+      <x:c r="G4" s="36" t="str">
+        <x:v>공식 후보 확인·시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H4" s="36" t="str">
+        <x:v>https://www.ine.gob.bo/index.php/estadisticas-economicas/construccion/indice-de-costo-de-la-construccio/</x:v>
+      </x:c>
+      <x:c r="I4" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J4" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K4" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L4" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M4" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N4" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O4" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P4" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q4" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R4" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S4" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/BOL/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T4" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="33" t="str">
+        <x:v>Cambodia</x:v>
+      </x:c>
+      <x:c r="B5" s="33" t="str">
+        <x:v>KHM</x:v>
+      </x:c>
+      <x:c r="C5" s="33" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D5" s="33" t="str"/>
+      <x:c r="E5" s="36" t="str"/>
+      <x:c r="F5" s="36" t="str">
+        <x:v>National Institute of Statistics</x:v>
+      </x:c>
+      <x:c r="G5" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H5" s="36" t="str">
+        <x:v>https://nis.gov.kh/</x:v>
+      </x:c>
+      <x:c r="I5" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J5" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K5" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L5" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M5" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N5" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O5" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P5" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q5" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R5" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S5" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/KHM/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T5" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="33" t="str">
+        <x:v>Côte d’Ivoire</x:v>
+      </x:c>
+      <x:c r="B6" s="33" t="str">
+        <x:v>CIV</x:v>
+      </x:c>
+      <x:c r="C6" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E6" s="36" t="str">
+        <x:v>Banque de Données des Prix de Référence—travaux</x:v>
+      </x:c>
+      <x:c r="F6" s="36" t="str">
+        <x:v>Direction Générale des Marchés Publics</x:v>
+      </x:c>
+      <x:c r="G6" s="36" t="str">
+        <x:v>공종 기준가격 후보·공개 시계열 미확인</x:v>
+      </x:c>
+      <x:c r="H6" s="36" t="str">
+        <x:v>https://bdpr.finances.gouv.ci/bdpr2023/accueil?p=presentation</x:v>
+      </x:c>
+      <x:c r="I6" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J6" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K6" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L6" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M6" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N6" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O6" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P6" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q6" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R6" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S6" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/CIV/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T6" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="33" t="str">
+        <x:v>Dominican Republic</x:v>
+      </x:c>
+      <x:c r="B7" s="33" t="str">
+        <x:v>DOM</x:v>
+      </x:c>
+      <x:c r="C7" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D7" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="36" t="str">
+        <x:v>Índice de Costos Directos de la Construcción de Viviendas (ICDV)</x:v>
+      </x:c>
+      <x:c r="F7" s="36" t="str">
+        <x:v>Oficina Nacional de Estadística</x:v>
+      </x:c>
+      <x:c r="G7" s="36" t="str">
+        <x:v>공식 후보 확인·주거 범위·시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H7" s="36" t="str">
+        <x:v>https://www.one.gob.do/publicaciones/2026/indice-de-costos-directos-de-la-construccion-de-viviendas-icdv-diciembre-2025/</x:v>
+      </x:c>
+      <x:c r="I7" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J7" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K7" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L7" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M7" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N7" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O7" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P7" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q7" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R7" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S7" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/DOM/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T7" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="33" t="str">
+        <x:v>Ecuador</x:v>
+      </x:c>
+      <x:c r="B8" s="33" t="str">
+        <x:v>ECU</x:v>
+      </x:c>
+      <x:c r="C8" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D8" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E8" s="36" t="str">
+        <x:v>Índice de Precios de la Construcción (IPCO)</x:v>
+      </x:c>
+      <x:c r="F8" s="36" t="str">
+        <x:v>Instituto Nacional de Estadística y Censos</x:v>
+      </x:c>
+      <x:c r="G8" s="36" t="str">
+        <x:v>공식 자재·장비 지수 확인·시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H8" s="36" t="str">
+        <x:v>https://www.ecuadorencifras.gob.ec/indice-de-precios-de-la-construccion/</x:v>
+      </x:c>
+      <x:c r="I8" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J8" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K8" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L8" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M8" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N8" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O8" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P8" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q8" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R8" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S8" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/ECU/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T8" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="33" t="str">
+        <x:v>El Salvador</x:v>
+      </x:c>
+      <x:c r="B9" s="33" t="str">
+        <x:v>SLV</x:v>
+      </x:c>
+      <x:c r="C9" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D9" s="33" t="str"/>
+      <x:c r="E9" s="36" t="str"/>
+      <x:c r="F9" s="36" t="str">
+        <x:v>Oficina Nacional de Estadística y Censos</x:v>
+      </x:c>
+      <x:c r="G9" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H9" s="36" t="str">
+        <x:v>https://onec.bcr.gob.sv/</x:v>
+      </x:c>
+      <x:c r="I9" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J9" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K9" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L9" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M9" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N9" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O9" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P9" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q9" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R9" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S9" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/SLV/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T9" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="33" t="str">
+        <x:v>Ethiopia</x:v>
+      </x:c>
+      <x:c r="B10" s="33" t="str">
+        <x:v>ETH</x:v>
+      </x:c>
+      <x:c r="C10" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D10" s="33" t="str"/>
+      <x:c r="E10" s="36" t="str"/>
+      <x:c r="F10" s="36" t="str">
+        <x:v>Ethiopian Statistics Service</x:v>
+      </x:c>
+      <x:c r="G10" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H10" s="36" t="str">
+        <x:v>https://ess.gov.et/price/</x:v>
+      </x:c>
+      <x:c r="I10" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J10" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K10" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L10" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M10" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N10" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O10" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P10" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q10" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R10" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S10" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/ETH/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T10" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="33" t="str">
+        <x:v>Fiji</x:v>
+      </x:c>
+      <x:c r="B11" s="33" t="str">
+        <x:v>FJI</x:v>
+      </x:c>
+      <x:c r="C11" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D11" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E11" s="36" t="str">
+        <x:v>Building Material Price Index (BMPI)</x:v>
+      </x:c>
+      <x:c r="F11" s="36" t="str">
+        <x:v>Fiji Bureau of Statistics</x:v>
+      </x:c>
+      <x:c r="G11" s="36" t="str">
+        <x:v>실제 연간 시계열 적재</x:v>
+      </x:c>
+      <x:c r="H11" s="36" t="str">
+        <x:v>https://www.statsfiji.gov.fj/statistics/economic-statistics/prices/</x:v>
+      </x:c>
+      <x:c r="I11" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J11" s="36" t="str">
+        <x:v>construction_materials_ppi</x:v>
+      </x:c>
+      <x:c r="K11" s="36" t="str">
+        <x:v>All Items Building Material Price Index</x:v>
+      </x:c>
+      <x:c r="L11" s="36" t="str">
+        <x:v>Fiji Bureau of Statistics</x:v>
+      </x:c>
+      <x:c r="M11" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N11" s="48" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="O11" s="33" t="str">
+        <x:v>2019</x:v>
+      </x:c>
+      <x:c r="P11" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q11" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R11" s="51" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="S11" s="36" t="str">
+        <x:v>https://www.statsfiji.gov.fj/statistics/economic-statistics/prices/</x:v>
+      </x:c>
+      <x:c r="T11" s="36" t="str">
+        <x:v>공식 상위지수 실제값 적재; 대상일 관측값 존재 여부를 실행 시 재확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="33" t="str">
+        <x:v>Ghana</x:v>
+      </x:c>
+      <x:c r="B12" s="33" t="str">
+        <x:v>GHA</x:v>
+      </x:c>
+      <x:c r="C12" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D12" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E12" s="36" t="str">
+        <x:v>Construction Producer Price Index (C-PPI)</x:v>
+      </x:c>
+      <x:c r="F12" s="36" t="str">
+        <x:v>Ghana Statistical Service</x:v>
+      </x:c>
+      <x:c r="G12" s="36" t="str">
+        <x:v>공식 후보 확인·시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H12" s="36" t="str">
+        <x:v>https://statsghana.gov.gh/gssmain/fileUpload/Industry/August_PPI_Construction.pdf</x:v>
+      </x:c>
+      <x:c r="I12" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J12" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K12" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L12" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M12" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N12" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O12" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P12" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q12" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R12" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S12" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/GHA/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T12" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="33" t="str">
+        <x:v>Indonesia</x:v>
+      </x:c>
+      <x:c r="B13" s="33" t="str">
+        <x:v>IDN</x:v>
+      </x:c>
+      <x:c r="C13" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D13" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E13" s="36" t="str">
+        <x:v>Wholesale Price Index—Construction Materials</x:v>
+      </x:c>
+      <x:c r="F13" s="36" t="str">
+        <x:v>BPS-Statistics Indonesia</x:v>
+      </x:c>
+      <x:c r="G13" s="36" t="str">
+        <x:v>공식 후보 확인·기준연도 개편 연결 필요</x:v>
+      </x:c>
+      <x:c r="H13" s="36" t="str">
+        <x:v>https://www.bps.go.id/en/publication/2026/04/22/4b14ba643724ed678156917c/the-wholesale-price-indices-of-indonesia--2023-100--2025.html</x:v>
+      </x:c>
+      <x:c r="I13" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J13" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K13" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L13" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M13" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N13" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O13" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P13" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q13" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R13" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S13" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/IDN/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T13" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="33" t="str">
+        <x:v>Iraq</x:v>
+      </x:c>
+      <x:c r="B14" s="33" t="str">
+        <x:v>IRQ</x:v>
+      </x:c>
+      <x:c r="C14" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D14" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E14" s="36" t="str">
+        <x:v>Construction materials prices and workers' wages</x:v>
+      </x:c>
+      <x:c r="F14" s="36" t="str">
+        <x:v>Central Statistical Organization</x:v>
+      </x:c>
+      <x:c r="G14" s="36" t="str">
+        <x:v>공식 구성요소 확인·BOQ 가중치 필요</x:v>
+      </x:c>
+      <x:c r="H14" s="36" t="str">
+        <x:v>https://www.cosit.gov.iq/ar/constr-stat/constr-pr</x:v>
+      </x:c>
+      <x:c r="I14" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J14" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K14" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L14" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M14" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N14" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O14" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P14" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q14" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R14" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S14" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/IRQ/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T14" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="33" t="str">
+        <x:v>Jordan</x:v>
+      </x:c>
+      <x:c r="B15" s="33" t="str">
+        <x:v>JOR</x:v>
+      </x:c>
+      <x:c r="C15" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D15" s="33" t="str"/>
+      <x:c r="E15" s="36" t="str"/>
+      <x:c r="F15" s="36" t="str">
+        <x:v>Department of Statistics</x:v>
+      </x:c>
+      <x:c r="G15" s="36" t="str">
+        <x:v>WPI는 확인했으나 적격 건설 하위지수 미확인</x:v>
+      </x:c>
+      <x:c r="H15" s="36" t="str">
+        <x:v>https://dosweb.dos.gov.jo/economic/price-indices/table-price-indices/</x:v>
+      </x:c>
+      <x:c r="I15" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J15" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K15" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L15" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M15" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N15" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O15" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P15" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q15" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R15" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S15" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/JOR/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T15" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="33" t="str">
+        <x:v>Kenya</x:v>
+      </x:c>
+      <x:c r="B16" s="33" t="str">
+        <x:v>KEN</x:v>
+      </x:c>
+      <x:c r="C16" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D16" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="36" t="str">
+        <x:v>Construction Input Price Index—Building Cost Index</x:v>
+      </x:c>
+      <x:c r="F16" s="36" t="str">
+        <x:v>Kenya National Bureau of Statistics</x:v>
+      </x:c>
+      <x:c r="G16" s="36" t="str">
+        <x:v>공식 후보 확인·분기 시계열 통합 필요</x:v>
+      </x:c>
+      <x:c r="H16" s="36" t="str">
+        <x:v>https://www.knbs.or.ke/button/construction-input-pi/</x:v>
+      </x:c>
+      <x:c r="I16" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J16" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K16" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L16" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M16" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N16" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O16" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P16" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q16" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R16" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S16" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/KEN/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T16" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="33" t="str">
+        <x:v>Kyrgyzstan</x:v>
+      </x:c>
+      <x:c r="B17" s="33" t="str">
+        <x:v>KGZ</x:v>
+      </x:c>
+      <x:c r="C17" s="33" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D17" s="33" t="str"/>
+      <x:c r="E17" s="36" t="str"/>
+      <x:c r="F17" s="36" t="str">
+        <x:v>National Statistical Committee</x:v>
+      </x:c>
+      <x:c r="G17" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H17" s="36" t="str">
+        <x:v>https://stat.gov.kg/en/statistics/ceny-i-tarify/</x:v>
+      </x:c>
+      <x:c r="I17" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J17" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K17" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L17" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M17" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N17" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O17" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P17" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q17" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R17" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S17" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/KGZ/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T17" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="33" t="str">
+        <x:v>Laos</x:v>
+      </x:c>
+      <x:c r="B18" s="33" t="str">
+        <x:v>LAO</x:v>
+      </x:c>
+      <x:c r="C18" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D18" s="33" t="str"/>
+      <x:c r="E18" s="36" t="str"/>
+      <x:c r="F18" s="36" t="str">
+        <x:v>Lao Statistics Bureau</x:v>
+      </x:c>
+      <x:c r="G18" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H18" s="36" t="str">
+        <x:v>https://www.lsb.gov.la/</x:v>
+      </x:c>
+      <x:c r="I18" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J18" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K18" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L18" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M18" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N18" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O18" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P18" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q18" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R18" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S18" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/LAO/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T18" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="33" t="str">
+        <x:v>Mozambique</x:v>
+      </x:c>
+      <x:c r="B19" s="33" t="str">
+        <x:v>MOZ</x:v>
+      </x:c>
+      <x:c r="C19" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D19" s="33" t="str"/>
+      <x:c r="E19" s="36" t="str"/>
+      <x:c r="F19" s="36" t="str">
+        <x:v>Instituto Nacional de Estatística</x:v>
+      </x:c>
+      <x:c r="G19" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H19" s="36" t="str">
+        <x:v>https://ine.gov.mz/en/</x:v>
+      </x:c>
+      <x:c r="I19" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J19" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K19" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L19" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M19" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N19" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O19" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P19" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q19" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R19" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S19" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/MOZ/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T19" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="33" t="str">
+        <x:v>Myanmar</x:v>
+      </x:c>
+      <x:c r="B20" s="33" t="str">
+        <x:v>MMR</x:v>
+      </x:c>
+      <x:c r="C20" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D20" s="33" t="str"/>
+      <x:c r="E20" s="36" t="str"/>
+      <x:c r="F20" s="36" t="str">
+        <x:v>Central Statistical Organization</x:v>
+      </x:c>
+      <x:c r="G20" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H20" s="36" t="str">
+        <x:v>https://www.csostat.gov.mm/home/NSDP</x:v>
+      </x:c>
+      <x:c r="I20" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J20" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K20" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L20" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M20" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N20" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O20" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P20" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q20" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R20" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S20" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/MMR/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T20" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="33" t="str">
+        <x:v>Nepal</x:v>
+      </x:c>
+      <x:c r="B21" s="33" t="str">
+        <x:v>NPL</x:v>
+      </x:c>
+      <x:c r="C21" s="33" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D21" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="36" t="str">
+        <x:v>Input Price Index of Construction Sectors (IPICS)</x:v>
+      </x:c>
+      <x:c r="F21" s="36" t="str">
+        <x:v>National Statistics Office</x:v>
+      </x:c>
+      <x:c r="G21" s="36" t="str">
+        <x:v>FY 2025/26 Q2까지 실제 분기 시계열 적재·최신값 잠정</x:v>
+      </x:c>
+      <x:c r="H21" s="36" t="str">
+        <x:v>https://nsonepal.gov.np/content/13454/price-and-production-index---q2-082-83/</x:v>
+      </x:c>
+      <x:c r="I21" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J21" s="36" t="str">
+        <x:v>national_construction_price</x:v>
+      </x:c>
+      <x:c r="K21" s="36" t="str">
+        <x:v>Overall Input Price Index of Construction Sectors (Material &amp; Labour)</x:v>
+      </x:c>
+      <x:c r="L21" s="36" t="str">
+        <x:v>National Statistics Office, Government of Nepal</x:v>
+      </x:c>
+      <x:c r="M21" s="33" t="str">
+        <x:v>quarterly</x:v>
+      </x:c>
+      <x:c r="N21" s="48" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="O21" s="33" t="str">
+        <x:v>2015-Q3</x:v>
+      </x:c>
+      <x:c r="P21" s="33" t="str">
+        <x:v>2025-Q4</x:v>
+      </x:c>
+      <x:c r="Q21" s="36" t="str">
+        <x:v>provisional</x:v>
+      </x:c>
+      <x:c r="R21" s="51" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="S21" s="36" t="str">
+        <x:v>https://nsonepal.gov.np/content/13454/price-and-production-index---q2-082-83/</x:v>
+      </x:c>
+      <x:c r="T21" s="36" t="str">
+        <x:v>공식 상위지수 실제값 적재; 대상일 관측값 존재 여부를 실행 시 재확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="33" t="str">
+        <x:v>Pakistan</x:v>
+      </x:c>
+      <x:c r="B22" s="33" t="str">
+        <x:v>PAK</x:v>
+      </x:c>
+      <x:c r="C22" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D22" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E22" s="36" t="str">
+        <x:v>Urban/Rural Construction Items Prices</x:v>
+      </x:c>
+      <x:c r="F22" s="36" t="str">
+        <x:v>Pakistan Bureau of Statistics</x:v>
+      </x:c>
+      <x:c r="G22" s="36" t="str">
+        <x:v>공식 구성요소 가격 확인·BOQ 가중치 필요</x:v>
+      </x:c>
+      <x:c r="H22" s="36" t="str">
+        <x:v>https://www.pbs.gov.pk/price-statistics/</x:v>
+      </x:c>
+      <x:c r="I22" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J22" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K22" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L22" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M22" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N22" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O22" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P22" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q22" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R22" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S22" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/PAK/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T22" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="33" t="str">
+        <x:v>Paraguay</x:v>
+      </x:c>
+      <x:c r="B23" s="33" t="str">
+        <x:v>PRY</x:v>
+      </x:c>
+      <x:c r="C23" s="33" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D23" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E23" s="36" t="str">
+        <x:v>CAPACO construction input and work-item costs</x:v>
+      </x:c>
+      <x:c r="F23" s="36" t="str">
+        <x:v>Cámara Paraguaya de la Industria de la Construcción</x:v>
+      </x:c>
+      <x:c r="G23" s="36" t="str">
+        <x:v>비정부 공종비 후보·공식 종합지수 미확인</x:v>
+      </x:c>
+      <x:c r="H23" s="36" t="str">
+        <x:v>https://www.capaco.org.py/</x:v>
+      </x:c>
+      <x:c r="I23" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J23" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K23" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L23" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M23" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N23" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O23" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P23" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q23" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R23" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S23" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/PRY/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T23" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="33" t="str">
+        <x:v>Philippines</x:v>
+      </x:c>
+      <x:c r="B24" s="33" t="str">
+        <x:v>PHL</x:v>
+      </x:c>
+      <x:c r="C24" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D24" s="33" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E24" s="36" t="str">
+        <x:v>Construction Materials Wholesale Price Index</x:v>
+      </x:c>
+      <x:c r="F24" s="36" t="str">
+        <x:v>Philippine Statistics Authority</x:v>
+      </x:c>
+      <x:c r="G24" s="36" t="str">
+        <x:v>공식 후보 확인·NCR 지역 범위·시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H24" s="36" t="str">
+        <x:v>https://psa.gov.ph/price-indices/cmwpi</x:v>
+      </x:c>
+      <x:c r="I24" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J24" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K24" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L24" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M24" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N24" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O24" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P24" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q24" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R24" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S24" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/PHL/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T24" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="33" t="str">
+        <x:v>Senegal</x:v>
+      </x:c>
+      <x:c r="B25" s="33" t="str">
+        <x:v>SEN</x:v>
+      </x:c>
+      <x:c r="C25" s="33" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D25" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" s="36" t="str">
+        <x:v>Indice des Coûts des BTP (IBTP)</x:v>
+      </x:c>
+      <x:c r="F25" s="36" t="str">
+        <x:v>Agence Nationale de la Statistique et de la Démographie</x:v>
+      </x:c>
+      <x:c r="G25" s="36" t="str">
+        <x:v>공식 후보 확인·2022Q4 신기준 연결 필요</x:v>
+      </x:c>
+      <x:c r="H25" s="36" t="str">
+        <x:v>https://www.ansd.sn/Indicateur/indice-des-couts-des-btp-ibtp</x:v>
+      </x:c>
+      <x:c r="I25" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J25" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K25" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L25" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M25" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N25" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O25" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P25" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q25" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R25" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S25" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/SEN/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T25" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="33" t="str">
+        <x:v>Sri Lanka</x:v>
+      </x:c>
+      <x:c r="B26" s="33" t="str">
+        <x:v>LKA</x:v>
+      </x:c>
+      <x:c r="C26" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D26" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="36" t="str">
+        <x:v>Cost of Construction Index</x:v>
+      </x:c>
+      <x:c r="F26" s="36" t="str">
+        <x:v>Construction Industry Development Authority</x:v>
+      </x:c>
+      <x:c r="G26" s="36" t="str">
+        <x:v>공식 자료에서 지수 존재 확인·원시 시계열 미적재</x:v>
+      </x:c>
+      <x:c r="H26" s="36" t="str">
+        <x:v>https://www.cbsl.gov.lk/sites/default/files/cbslweb_documents/publications/otherpub/publication_sri_lanka_socio_economic_data_folder_2025_e.pdf</x:v>
+      </x:c>
+      <x:c r="I26" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J26" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K26" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L26" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M26" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N26" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O26" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P26" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q26" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R26" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S26" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/LKA/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T26" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="33" t="str">
+        <x:v>Timor-Leste</x:v>
+      </x:c>
+      <x:c r="B27" s="33" t="str">
+        <x:v>TLS</x:v>
+      </x:c>
+      <x:c r="C27" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D27" s="33" t="str"/>
+      <x:c r="E27" s="36" t="str"/>
+      <x:c r="F27" s="36" t="str">
+        <x:v>Instituto Nacional de Estatística Timor-Leste</x:v>
+      </x:c>
+      <x:c r="G27" s="36" t="str">
+        <x:v>공개된 적격 건설지수 미확인</x:v>
+      </x:c>
+      <x:c r="H27" s="36" t="str">
+        <x:v>https://inetl-ip.gov.tl/</x:v>
+      </x:c>
+      <x:c r="I27" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J27" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K27" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L27" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M27" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N27" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O27" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P27" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q27" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R27" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S27" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/TLS/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T27" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="33" t="str">
+        <x:v>Turkmenistan</x:v>
+      </x:c>
+      <x:c r="B28" s="33" t="str">
+        <x:v>TKM</x:v>
+      </x:c>
+      <x:c r="C28" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D28" s="33" t="str"/>
+      <x:c r="E28" s="36" t="str"/>
+      <x:c r="F28" s="36" t="str">
+        <x:v>State Committee of Turkmenistan on Statistics</x:v>
+      </x:c>
+      <x:c r="G28" s="36" t="str">
+        <x:v>건설 가격정보 시스템 추진은 확인했으나 공개 시계열 미확인</x:v>
+      </x:c>
+      <x:c r="H28" s="36" t="str">
+        <x:v>https://stat.gov.tm/en/</x:v>
+      </x:c>
+      <x:c r="I28" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J28" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K28" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L28" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M28" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N28" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O28" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P28" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q28" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R28" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S28" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/TKM/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T28" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="33" t="str">
+        <x:v>Uganda</x:v>
+      </x:c>
+      <x:c r="B29" s="33" t="str">
+        <x:v>UGA</x:v>
+      </x:c>
+      <x:c r="C29" s="33" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D29" s="33" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E29" s="36" t="str">
+        <x:v>Construction Input Price Index (CIPI)</x:v>
+      </x:c>
+      <x:c r="F29" s="36" t="str">
+        <x:v>Uganda Bureau of Statistics</x:v>
+      </x:c>
+      <x:c r="G29" s="36" t="str">
+        <x:v>공식 후보 확인·월별 시계열 통합 필요</x:v>
+      </x:c>
+      <x:c r="H29" s="36" t="str">
+        <x:v>https://www.ubos.org/?p_id=104&amp;pagename=explore-publications</x:v>
+      </x:c>
+      <x:c r="I29" s="33" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="J29" s="36" t="str">
+        <x:v>gdp_deflator</x:v>
+      </x:c>
+      <x:c r="K29" s="36" t="str">
+        <x:v>GDP deflator (base year varies by country)</x:v>
+      </x:c>
+      <x:c r="L29" s="36" t="str">
+        <x:v>World Bank, World Development Indicators</x:v>
+      </x:c>
+      <x:c r="M29" s="33" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N29" s="48" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O29" s="33" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P29" s="33" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q29" s="36" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R29" s="51" t="n">
+        <x:v>46232.95527777778</x:v>
+      </x:c>
+      <x:c r="S29" s="36" t="str">
+        <x:v>https://api.worldbank.org/v2/country/UGA/indicator/NY.GDP.DEFL.ZS</x:v>
+      </x:c>
+      <x:c r="T29" s="36" t="str">
+        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="34" t="str">
+        <x:v>Uzbekistan</x:v>
+      </x:c>
+      <x:c r="B30" s="34" t="str">
+        <x:v>UZB</x:v>
+      </x:c>
+      <x:c r="C30" s="34" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D30" s="34" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E30" s="37" t="str">
+        <x:v>Price index for investments in fixed assets and construction works</x:v>
+      </x:c>
+      <x:c r="F30" s="37" t="str">
+        <x:v>National Statistics Committee</x:v>
+      </x:c>
+      <x:c r="G30" s="37" t="str">
+        <x:v>실제 연간 시계열 적재·범위 주의</x:v>
+      </x:c>
+      <x:c r="H30" s="37" t="str">
+        <x:v>https://siat.stat.uz/data/1302/?lang=en</x:v>
+      </x:c>
+      <x:c r="I30" s="34" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J30" s="37" t="str">
+        <x:v>national_construction_price</x:v>
+      </x:c>
+      <x:c r="K30" s="37" t="str">
+        <x:v>Price index for investments in fixed assets and construction works</x:v>
+      </x:c>
+      <x:c r="L30" s="37" t="str">
+        <x:v>National Statistics Committee of the Republic of Uzbekistan</x:v>
+      </x:c>
+      <x:c r="M30" s="34" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="N30" s="49" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O30" s="34" t="str">
+        <x:v>2015</x:v>
+      </x:c>
+      <x:c r="P30" s="34" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="Q30" s="37" t="str">
+        <x:v>published</x:v>
+      </x:c>
+      <x:c r="R30" s="52" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="S30" s="37" t="str">
+        <x:v>https://siat.stat.uz/data/1302/?lang=en</x:v>
+      </x:c>
+      <x:c r="T30" s="37" t="str">
+        <x:v>공식 상위지수 실제값 적재; 대상일 관측값 존재 여부를 실행 시 재확인</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:T1"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="Q3:Q30">
+    <x:cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="provisional"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2e3ebfb67d1446a"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7779,34 +9661,78 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="33" t="str">
-        <x:v>v_sample_coverage</x:v>
+        <x:v>price_index_sources</x:v>
       </x:c>
       <x:c r="B12" s="36" t="str">
-        <x:v>국가×시설×유형 표본수와 명목범위</x:v>
+        <x:v>국가별 가격지수 출처·범위·우선순위</x:v>
       </x:c>
       <x:c r="C12" s="36" t="str">
-        <x:v>조회용 VIEW</x:v>
+        <x:v>source_id</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="33" t="str">
+        <x:v>price_index_values</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
+        <x:v>분석용 기간·원래 기간·값·잠정/수정 상태·공개 URL</x:v>
+      </x:c>
+      <x:c r="C13" s="36" t="str">
+        <x:v>source_id, period</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="33" t="str">
+        <x:v>v_price_index_coverage</x:v>
+      </x:c>
+      <x:c r="B14" s="36" t="str">
+        <x:v>국가·지수별 실제 관측기간과 최신값 상태</x:v>
+      </x:c>
+      <x:c r="C14" s="36" t="str">
+        <x:v>조회용 VIEW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="33" t="str">
+        <x:v>v_best_available_price_index</x:v>
+      </x:c>
+      <x:c r="B15" s="36" t="str">
+        <x:v>국가별 현재 선택 가능한 최고 우선순위 실제 지수</x:v>
+      </x:c>
+      <x:c r="C15" s="36" t="str">
+        <x:v>조회용 VIEW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="33" t="str">
+        <x:v>v_sample_coverage</x:v>
+      </x:c>
+      <x:c r="B16" s="36" t="str">
+        <x:v>국가×시설×유형 표본수와 명목범위</x:v>
+      </x:c>
+      <x:c r="C16" s="36" t="str">
+        <x:v>조회용 VIEW</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="33" t="str">
         <x:v>v_yearly_inventory</x:v>
       </x:c>
-      <x:c r="B13" s="36" t="str">
+      <x:c r="B17" s="36" t="str">
         <x:v>연도별 검토사례·미보정 건수</x:v>
       </x:c>
-      <x:c r="C13" s="36" t="str">
+      <x:c r="C17" s="36" t="str">
         <x:v>조회용 VIEW</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="34" t="str">
+    <x:row r="18">
+      <x:c r="A18" s="34" t="str">
         <x:v>v_duplicate_attachments</x:v>
       </x:c>
-      <x:c r="B14" s="37" t="str">
+      <x:c r="B18" s="37" t="str">
         <x:v>동일 SHA-256 첨부파일</x:v>
       </x:c>
-      <x:c r="C14" s="37" t="str">
+      <x:c r="C18" s="37" t="str">
         <x:v>조회용 VIEW</x:v>
       </x:c>
     </x:row>
@@ -7816,12 +9742,12 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0879c92fe50401a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa82d875f97b415c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7844,41 +9770,57 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="32" t="str">
-        <x:v>유사사례 검색</x:v>
+        <x:v>국가·시설 유사사례</x:v>
       </x:c>
       <x:c r="B3" s="35" t="str">
-        <x:v>SELECT * FROM reviewed_cases WHERE country = 'Nepal' AND work_type LIKE '%신축%' ORDER BY notice_date DESC;</x:v>
+        <x:v>WITH p(country_name, facility_keyword) AS (VALUES ('Nepal','교육')) SELECT r.* FROM reviewed_cases r CROSS JOIN p WHERE r.country=p.country_name ORDER BY CASE WHEN r.facility_type LIKE '%'||p.facility_keyword||'%' THEN 0 ELSE 1 END, r.notice_date DESC;</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="33" t="str">
-        <x:v>표본수 확인</x:v>
+        <x:v>국가별 표본수</x:v>
       </x:c>
       <x:c r="B4" s="36" t="str">
-        <x:v>SELECT * FROM v_sample_coverage WHERE country = 'Nepal' ORDER BY reviewed_case_count DESC;</x:v>
+        <x:v>WITH p(country_name) AS (VALUES ('Nepal')) SELECT c.* FROM v_sample_coverage c CROSS JOIN p WHERE c.country=p.country_name ORDER BY reviewed_case_count DESC;</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="33" t="str">
-        <x:v>근거 추적</x:v>
+        <x:v>국가별 지수 선택</x:v>
       </x:c>
       <x:c r="B5" s="36" t="str">
-        <x:v>SELECT category, source_file, source_locator, evidence_text FROM evidence WHERE bid_no = 'L2022-00029-1';</x:v>
+        <x:v>WITH p(country_name) AS (VALUES ('Nepal')) SELECT b.* FROM v_best_available_price_index b CROSS JOIN p WHERE b.country=p.country_name;</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="33" t="str">
+        <x:v>지수 원래 기간·상태</x:v>
+      </x:c>
+      <x:c r="B6" s="36" t="str">
+        <x:v>SELECT period, native_period, value, observation_status, release_url, retrieved_at FROM price_index_values WHERE source_id='NSO_NPL_IPICS_OVERALL' ORDER BY period;</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="33" t="str">
+        <x:v>근거 추적</x:v>
+      </x:c>
+      <x:c r="B7" s="36" t="str">
+        <x:v>SELECT category, source_file, source_locator, evidence_text FROM evidence WHERE bid_no = '&lt;공고번호&gt;';</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="33" t="str">
         <x:v>첨부 확인</x:v>
       </x:c>
-      <x:c r="B6" s="36" t="str">
-        <x:v>SELECT original_name, bytes, sha256, relative_path FROM attachments WHERE bid_no = 'L2022-00029-1';</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="34" t="str">
+      <x:c r="B8" s="36" t="str">
+        <x:v>SELECT original_name, bytes, sha256, relative_path FROM attachments WHERE bid_no = '&lt;공고번호&gt;';</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="34" t="str">
         <x:v>연도별 현황</x:v>
       </x:c>
-      <x:c r="B7" s="37" t="str">
+      <x:c r="B9" s="37" t="str">
         <x:v>SELECT * FROM v_yearly_inventory ORDER BY notice_year;</x:v>
       </x:c>
     </x:row>
@@ -7888,7 +9830,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R652d7198260c4f06"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd33f14f98d84534"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: audit KOICA-only construction cost evidence
</commit_message>
<xml_diff>
--- a/outputs/koica-construction-distribution/KOICA_건축사업_사례라이브러리_2016-2025.xlsx
+++ b/outputs/koica-construction-distribution/KOICA_건축사업_사례라이브러리_2016-2025.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Rda15b7a2987a48aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검토사례" sheetId="2" r:id="Ra2c5b37405684bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="표본현황" sheetId="3" r:id="R8ee6e73d65c6424b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="국가지수현황" sheetId="4" r:id="R03fae5b2d6a645f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터사전" sheetId="5" r:id="R5c42feaf85534f91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL 예시" sheetId="6" r:id="Rad8ded3cd6ef4ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용안내" sheetId="1" r:id="Rae5a76be28854f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검토사례" sheetId="2" r:id="R51e5258edaea4b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="표본현황" sheetId="3" r:id="Ra388f1d020c54d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="국가지수현황" sheetId="4" r:id="R891a9068855b46e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="데이터사전" sheetId="5" r:id="R20ee0870d7794c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SQL 예시" sheetId="6" r:id="R77d66ce56b0c46ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -305,7 +305,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{C51560CE-245F-46B0-A622-F8E49E70857B}"/>
+  <xltc:person displayName="User" id="{C38325F0-187D-4497-ADE0-FE47D0103855}"/>
 </xltc:personList>
 </file>
 
@@ -620,7 +620,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="7" t="str">
-        <x:v>이 파일은 사례 열람용입니다. 원본 데이터는 SQLite이며, 여기에 미래 사업 권고단가는 없습니다.</x:v>
+        <x:v>이 파일은 KOICA 사례 열람용입니다. 외부 공여기관 자료는 포함하지 않으며, 미래 사업 권고단가도 제공하지 않습니다.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -5414,7 +5414,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b69f1a8c9724e2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc30f6f5a38b461d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7727,7 +7727,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93046aa8c2f34a0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda7f7a9dc35246d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7760,7 +7760,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="25" t="str">
-        <x:v>28개국 가격지수 후보·현재 선택·관측상태</x:v>
+        <x:v>28개국 국가 공식 가격지수 후보·적재·관측상태</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
@@ -7850,41 +7850,19 @@
       <x:c r="H3" s="35" t="str">
         <x:v>https://bbs.gov.bd/site/page/29b379ff-7bac-41d9-b321-e41929bab4a1</x:v>
       </x:c>
-      <x:c r="I3" s="32" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J3" s="35" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K3" s="35" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L3" s="35" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M3" s="32" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N3" s="47" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O3" s="32" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P3" s="32" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q3" s="35" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R3" s="50" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S3" s="35" t="str">
-        <x:v>https://api.worldbank.org/v2/country/BGD/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I3" s="32" t="str"/>
+      <x:c r="J3" s="35" t="str"/>
+      <x:c r="K3" s="35" t="str"/>
+      <x:c r="L3" s="35" t="str"/>
+      <x:c r="M3" s="32" t="str"/>
+      <x:c r="N3" s="47" t="str"/>
+      <x:c r="O3" s="32" t="str"/>
+      <x:c r="P3" s="32" t="str"/>
+      <x:c r="Q3" s="35" t="str"/>
+      <x:c r="R3" s="50" t="str"/>
+      <x:c r="S3" s="35" t="str"/>
       <x:c r="T3" s="35" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -7912,41 +7890,19 @@
       <x:c r="H4" s="36" t="str">
         <x:v>https://www.ine.gob.bo/index.php/estadisticas-economicas/construccion/indice-de-costo-de-la-construccio/</x:v>
       </x:c>
-      <x:c r="I4" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J4" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K4" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L4" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M4" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N4" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O4" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P4" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q4" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R4" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S4" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/BOL/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I4" s="33" t="str"/>
+      <x:c r="J4" s="36" t="str"/>
+      <x:c r="K4" s="36" t="str"/>
+      <x:c r="L4" s="36" t="str"/>
+      <x:c r="M4" s="33" t="str"/>
+      <x:c r="N4" s="48" t="str"/>
+      <x:c r="O4" s="33" t="str"/>
+      <x:c r="P4" s="33" t="str"/>
+      <x:c r="Q4" s="36" t="str"/>
+      <x:c r="R4" s="51" t="str"/>
+      <x:c r="S4" s="36" t="str"/>
       <x:c r="T4" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -7970,41 +7926,19 @@
       <x:c r="H5" s="36" t="str">
         <x:v>https://nis.gov.kh/</x:v>
       </x:c>
-      <x:c r="I5" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J5" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K5" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L5" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M5" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N5" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O5" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P5" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q5" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R5" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S5" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/KHM/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I5" s="33" t="str"/>
+      <x:c r="J5" s="36" t="str"/>
+      <x:c r="K5" s="36" t="str"/>
+      <x:c r="L5" s="36" t="str"/>
+      <x:c r="M5" s="33" t="str"/>
+      <x:c r="N5" s="48" t="str"/>
+      <x:c r="O5" s="33" t="str"/>
+      <x:c r="P5" s="33" t="str"/>
+      <x:c r="Q5" s="36" t="str"/>
+      <x:c r="R5" s="51" t="str"/>
+      <x:c r="S5" s="36" t="str"/>
       <x:c r="T5" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -8032,41 +7966,19 @@
       <x:c r="H6" s="36" t="str">
         <x:v>https://bdpr.finances.gouv.ci/bdpr2023/accueil?p=presentation</x:v>
       </x:c>
-      <x:c r="I6" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J6" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K6" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L6" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M6" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N6" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O6" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P6" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q6" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R6" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S6" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/CIV/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I6" s="33" t="str"/>
+      <x:c r="J6" s="36" t="str"/>
+      <x:c r="K6" s="36" t="str"/>
+      <x:c r="L6" s="36" t="str"/>
+      <x:c r="M6" s="33" t="str"/>
+      <x:c r="N6" s="48" t="str"/>
+      <x:c r="O6" s="33" t="str"/>
+      <x:c r="P6" s="33" t="str"/>
+      <x:c r="Q6" s="36" t="str"/>
+      <x:c r="R6" s="51" t="str"/>
+      <x:c r="S6" s="36" t="str"/>
       <x:c r="T6" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -8094,41 +8006,19 @@
       <x:c r="H7" s="36" t="str">
         <x:v>https://www.one.gob.do/publicaciones/2026/indice-de-costos-directos-de-la-construccion-de-viviendas-icdv-diciembre-2025/</x:v>
       </x:c>
-      <x:c r="I7" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J7" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K7" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L7" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M7" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N7" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O7" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P7" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q7" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R7" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S7" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/DOM/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I7" s="33" t="str"/>
+      <x:c r="J7" s="36" t="str"/>
+      <x:c r="K7" s="36" t="str"/>
+      <x:c r="L7" s="36" t="str"/>
+      <x:c r="M7" s="33" t="str"/>
+      <x:c r="N7" s="48" t="str"/>
+      <x:c r="O7" s="33" t="str"/>
+      <x:c r="P7" s="33" t="str"/>
+      <x:c r="Q7" s="36" t="str"/>
+      <x:c r="R7" s="51" t="str"/>
+      <x:c r="S7" s="36" t="str"/>
       <x:c r="T7" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -8156,41 +8046,19 @@
       <x:c r="H8" s="36" t="str">
         <x:v>https://www.ecuadorencifras.gob.ec/indice-de-precios-de-la-construccion/</x:v>
       </x:c>
-      <x:c r="I8" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J8" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K8" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L8" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M8" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N8" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O8" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P8" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q8" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R8" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S8" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/ECU/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I8" s="33" t="str"/>
+      <x:c r="J8" s="36" t="str"/>
+      <x:c r="K8" s="36" t="str"/>
+      <x:c r="L8" s="36" t="str"/>
+      <x:c r="M8" s="33" t="str"/>
+      <x:c r="N8" s="48" t="str"/>
+      <x:c r="O8" s="33" t="str"/>
+      <x:c r="P8" s="33" t="str"/>
+      <x:c r="Q8" s="36" t="str"/>
+      <x:c r="R8" s="51" t="str"/>
+      <x:c r="S8" s="36" t="str"/>
       <x:c r="T8" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -8214,41 +8082,19 @@
       <x:c r="H9" s="36" t="str">
         <x:v>https://onec.bcr.gob.sv/</x:v>
       </x:c>
-      <x:c r="I9" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J9" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K9" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L9" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M9" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N9" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O9" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P9" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q9" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R9" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S9" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/SLV/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I9" s="33" t="str"/>
+      <x:c r="J9" s="36" t="str"/>
+      <x:c r="K9" s="36" t="str"/>
+      <x:c r="L9" s="36" t="str"/>
+      <x:c r="M9" s="33" t="str"/>
+      <x:c r="N9" s="48" t="str"/>
+      <x:c r="O9" s="33" t="str"/>
+      <x:c r="P9" s="33" t="str"/>
+      <x:c r="Q9" s="36" t="str"/>
+      <x:c r="R9" s="51" t="str"/>
+      <x:c r="S9" s="36" t="str"/>
       <x:c r="T9" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -8272,41 +8118,19 @@
       <x:c r="H10" s="36" t="str">
         <x:v>https://ess.gov.et/price/</x:v>
       </x:c>
-      <x:c r="I10" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J10" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K10" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L10" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M10" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N10" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O10" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P10" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q10" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R10" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S10" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/ETH/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I10" s="33" t="str"/>
+      <x:c r="J10" s="36" t="str"/>
+      <x:c r="K10" s="36" t="str"/>
+      <x:c r="L10" s="36" t="str"/>
+      <x:c r="M10" s="33" t="str"/>
+      <x:c r="N10" s="48" t="str"/>
+      <x:c r="O10" s="33" t="str"/>
+      <x:c r="P10" s="33" t="str"/>
+      <x:c r="Q10" s="36" t="str"/>
+      <x:c r="R10" s="51" t="str"/>
+      <x:c r="S10" s="36" t="str"/>
       <x:c r="T10" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -8396,41 +8220,19 @@
       <x:c r="H12" s="36" t="str">
         <x:v>https://statsghana.gov.gh/gssmain/fileUpload/Industry/August_PPI_Construction.pdf</x:v>
       </x:c>
-      <x:c r="I12" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J12" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K12" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L12" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M12" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N12" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O12" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P12" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q12" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R12" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S12" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/GHA/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I12" s="33" t="str"/>
+      <x:c r="J12" s="36" t="str"/>
+      <x:c r="K12" s="36" t="str"/>
+      <x:c r="L12" s="36" t="str"/>
+      <x:c r="M12" s="33" t="str"/>
+      <x:c r="N12" s="48" t="str"/>
+      <x:c r="O12" s="33" t="str"/>
+      <x:c r="P12" s="33" t="str"/>
+      <x:c r="Q12" s="36" t="str"/>
+      <x:c r="R12" s="51" t="str"/>
+      <x:c r="S12" s="36" t="str"/>
       <x:c r="T12" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -8458,41 +8260,19 @@
       <x:c r="H13" s="36" t="str">
         <x:v>https://www.bps.go.id/en/publication/2026/04/22/4b14ba643724ed678156917c/the-wholesale-price-indices-of-indonesia--2023-100--2025.html</x:v>
       </x:c>
-      <x:c r="I13" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J13" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K13" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L13" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M13" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N13" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O13" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P13" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q13" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R13" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S13" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/IDN/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I13" s="33" t="str"/>
+      <x:c r="J13" s="36" t="str"/>
+      <x:c r="K13" s="36" t="str"/>
+      <x:c r="L13" s="36" t="str"/>
+      <x:c r="M13" s="33" t="str"/>
+      <x:c r="N13" s="48" t="str"/>
+      <x:c r="O13" s="33" t="str"/>
+      <x:c r="P13" s="33" t="str"/>
+      <x:c r="Q13" s="36" t="str"/>
+      <x:c r="R13" s="51" t="str"/>
+      <x:c r="S13" s="36" t="str"/>
       <x:c r="T13" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -8520,41 +8300,19 @@
       <x:c r="H14" s="36" t="str">
         <x:v>https://www.cosit.gov.iq/ar/constr-stat/constr-pr</x:v>
       </x:c>
-      <x:c r="I14" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J14" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K14" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L14" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M14" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N14" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O14" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P14" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q14" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R14" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S14" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/IRQ/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I14" s="33" t="str"/>
+      <x:c r="J14" s="36" t="str"/>
+      <x:c r="K14" s="36" t="str"/>
+      <x:c r="L14" s="36" t="str"/>
+      <x:c r="M14" s="33" t="str"/>
+      <x:c r="N14" s="48" t="str"/>
+      <x:c r="O14" s="33" t="str"/>
+      <x:c r="P14" s="33" t="str"/>
+      <x:c r="Q14" s="36" t="str"/>
+      <x:c r="R14" s="51" t="str"/>
+      <x:c r="S14" s="36" t="str"/>
       <x:c r="T14" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -8578,41 +8336,19 @@
       <x:c r="H15" s="36" t="str">
         <x:v>https://dosweb.dos.gov.jo/economic/price-indices/table-price-indices/</x:v>
       </x:c>
-      <x:c r="I15" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J15" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K15" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L15" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M15" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N15" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O15" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P15" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q15" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R15" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S15" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/JOR/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I15" s="33" t="str"/>
+      <x:c r="J15" s="36" t="str"/>
+      <x:c r="K15" s="36" t="str"/>
+      <x:c r="L15" s="36" t="str"/>
+      <x:c r="M15" s="33" t="str"/>
+      <x:c r="N15" s="48" t="str"/>
+      <x:c r="O15" s="33" t="str"/>
+      <x:c r="P15" s="33" t="str"/>
+      <x:c r="Q15" s="36" t="str"/>
+      <x:c r="R15" s="51" t="str"/>
+      <x:c r="S15" s="36" t="str"/>
       <x:c r="T15" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -8640,41 +8376,19 @@
       <x:c r="H16" s="36" t="str">
         <x:v>https://www.knbs.or.ke/button/construction-input-pi/</x:v>
       </x:c>
-      <x:c r="I16" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J16" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K16" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L16" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M16" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N16" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O16" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P16" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q16" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R16" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S16" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/KEN/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I16" s="33" t="str"/>
+      <x:c r="J16" s="36" t="str"/>
+      <x:c r="K16" s="36" t="str"/>
+      <x:c r="L16" s="36" t="str"/>
+      <x:c r="M16" s="33" t="str"/>
+      <x:c r="N16" s="48" t="str"/>
+      <x:c r="O16" s="33" t="str"/>
+      <x:c r="P16" s="33" t="str"/>
+      <x:c r="Q16" s="36" t="str"/>
+      <x:c r="R16" s="51" t="str"/>
+      <x:c r="S16" s="36" t="str"/>
       <x:c r="T16" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -8698,41 +8412,19 @@
       <x:c r="H17" s="36" t="str">
         <x:v>https://stat.gov.kg/en/statistics/ceny-i-tarify/</x:v>
       </x:c>
-      <x:c r="I17" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J17" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K17" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L17" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M17" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N17" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O17" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P17" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q17" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R17" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S17" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/KGZ/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I17" s="33" t="str"/>
+      <x:c r="J17" s="36" t="str"/>
+      <x:c r="K17" s="36" t="str"/>
+      <x:c r="L17" s="36" t="str"/>
+      <x:c r="M17" s="33" t="str"/>
+      <x:c r="N17" s="48" t="str"/>
+      <x:c r="O17" s="33" t="str"/>
+      <x:c r="P17" s="33" t="str"/>
+      <x:c r="Q17" s="36" t="str"/>
+      <x:c r="R17" s="51" t="str"/>
+      <x:c r="S17" s="36" t="str"/>
       <x:c r="T17" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -8756,41 +8448,19 @@
       <x:c r="H18" s="36" t="str">
         <x:v>https://www.lsb.gov.la/</x:v>
       </x:c>
-      <x:c r="I18" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J18" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K18" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L18" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M18" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N18" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O18" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P18" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q18" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R18" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S18" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/LAO/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I18" s="33" t="str"/>
+      <x:c r="J18" s="36" t="str"/>
+      <x:c r="K18" s="36" t="str"/>
+      <x:c r="L18" s="36" t="str"/>
+      <x:c r="M18" s="33" t="str"/>
+      <x:c r="N18" s="48" t="str"/>
+      <x:c r="O18" s="33" t="str"/>
+      <x:c r="P18" s="33" t="str"/>
+      <x:c r="Q18" s="36" t="str"/>
+      <x:c r="R18" s="51" t="str"/>
+      <x:c r="S18" s="36" t="str"/>
       <x:c r="T18" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -8814,41 +8484,19 @@
       <x:c r="H19" s="36" t="str">
         <x:v>https://ine.gov.mz/en/</x:v>
       </x:c>
-      <x:c r="I19" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J19" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K19" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L19" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M19" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N19" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O19" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P19" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q19" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R19" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S19" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/MOZ/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I19" s="33" t="str"/>
+      <x:c r="J19" s="36" t="str"/>
+      <x:c r="K19" s="36" t="str"/>
+      <x:c r="L19" s="36" t="str"/>
+      <x:c r="M19" s="33" t="str"/>
+      <x:c r="N19" s="48" t="str"/>
+      <x:c r="O19" s="33" t="str"/>
+      <x:c r="P19" s="33" t="str"/>
+      <x:c r="Q19" s="36" t="str"/>
+      <x:c r="R19" s="51" t="str"/>
+      <x:c r="S19" s="36" t="str"/>
       <x:c r="T19" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -8872,41 +8520,19 @@
       <x:c r="H20" s="36" t="str">
         <x:v>https://www.csostat.gov.mm/home/NSDP</x:v>
       </x:c>
-      <x:c r="I20" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J20" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K20" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L20" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M20" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N20" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O20" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P20" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q20" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R20" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S20" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/MMR/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I20" s="33" t="str"/>
+      <x:c r="J20" s="36" t="str"/>
+      <x:c r="K20" s="36" t="str"/>
+      <x:c r="L20" s="36" t="str"/>
+      <x:c r="M20" s="33" t="str"/>
+      <x:c r="N20" s="48" t="str"/>
+      <x:c r="O20" s="33" t="str"/>
+      <x:c r="P20" s="33" t="str"/>
+      <x:c r="Q20" s="36" t="str"/>
+      <x:c r="R20" s="51" t="str"/>
+      <x:c r="S20" s="36" t="str"/>
       <x:c r="T20" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -8996,41 +8622,19 @@
       <x:c r="H22" s="36" t="str">
         <x:v>https://www.pbs.gov.pk/price-statistics/</x:v>
       </x:c>
-      <x:c r="I22" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J22" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K22" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L22" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M22" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N22" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O22" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P22" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q22" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R22" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S22" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/PAK/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I22" s="33" t="str"/>
+      <x:c r="J22" s="36" t="str"/>
+      <x:c r="K22" s="36" t="str"/>
+      <x:c r="L22" s="36" t="str"/>
+      <x:c r="M22" s="33" t="str"/>
+      <x:c r="N22" s="48" t="str"/>
+      <x:c r="O22" s="33" t="str"/>
+      <x:c r="P22" s="33" t="str"/>
+      <x:c r="Q22" s="36" t="str"/>
+      <x:c r="R22" s="51" t="str"/>
+      <x:c r="S22" s="36" t="str"/>
       <x:c r="T22" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -9058,41 +8662,19 @@
       <x:c r="H23" s="36" t="str">
         <x:v>https://www.capaco.org.py/</x:v>
       </x:c>
-      <x:c r="I23" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J23" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K23" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L23" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M23" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N23" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O23" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P23" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q23" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R23" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S23" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/PRY/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I23" s="33" t="str"/>
+      <x:c r="J23" s="36" t="str"/>
+      <x:c r="K23" s="36" t="str"/>
+      <x:c r="L23" s="36" t="str"/>
+      <x:c r="M23" s="33" t="str"/>
+      <x:c r="N23" s="48" t="str"/>
+      <x:c r="O23" s="33" t="str"/>
+      <x:c r="P23" s="33" t="str"/>
+      <x:c r="Q23" s="36" t="str"/>
+      <x:c r="R23" s="51" t="str"/>
+      <x:c r="S23" s="36" t="str"/>
       <x:c r="T23" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -9120,41 +8702,19 @@
       <x:c r="H24" s="36" t="str">
         <x:v>https://psa.gov.ph/price-indices/cmwpi</x:v>
       </x:c>
-      <x:c r="I24" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J24" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K24" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L24" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M24" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N24" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O24" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P24" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q24" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R24" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S24" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/PHL/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I24" s="33" t="str"/>
+      <x:c r="J24" s="36" t="str"/>
+      <x:c r="K24" s="36" t="str"/>
+      <x:c r="L24" s="36" t="str"/>
+      <x:c r="M24" s="33" t="str"/>
+      <x:c r="N24" s="48" t="str"/>
+      <x:c r="O24" s="33" t="str"/>
+      <x:c r="P24" s="33" t="str"/>
+      <x:c r="Q24" s="36" t="str"/>
+      <x:c r="R24" s="51" t="str"/>
+      <x:c r="S24" s="36" t="str"/>
       <x:c r="T24" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -9182,41 +8742,19 @@
       <x:c r="H25" s="36" t="str">
         <x:v>https://www.ansd.sn/Indicateur/indice-des-couts-des-btp-ibtp</x:v>
       </x:c>
-      <x:c r="I25" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J25" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K25" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L25" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M25" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N25" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O25" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P25" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q25" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R25" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S25" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/SEN/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I25" s="33" t="str"/>
+      <x:c r="J25" s="36" t="str"/>
+      <x:c r="K25" s="36" t="str"/>
+      <x:c r="L25" s="36" t="str"/>
+      <x:c r="M25" s="33" t="str"/>
+      <x:c r="N25" s="48" t="str"/>
+      <x:c r="O25" s="33" t="str"/>
+      <x:c r="P25" s="33" t="str"/>
+      <x:c r="Q25" s="36" t="str"/>
+      <x:c r="R25" s="51" t="str"/>
+      <x:c r="S25" s="36" t="str"/>
       <x:c r="T25" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -9244,41 +8782,19 @@
       <x:c r="H26" s="36" t="str">
         <x:v>https://www.cbsl.gov.lk/sites/default/files/cbslweb_documents/publications/otherpub/publication_sri_lanka_socio_economic_data_folder_2025_e.pdf</x:v>
       </x:c>
-      <x:c r="I26" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J26" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K26" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L26" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M26" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N26" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O26" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P26" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q26" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R26" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S26" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/LKA/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I26" s="33" t="str"/>
+      <x:c r="J26" s="36" t="str"/>
+      <x:c r="K26" s="36" t="str"/>
+      <x:c r="L26" s="36" t="str"/>
+      <x:c r="M26" s="33" t="str"/>
+      <x:c r="N26" s="48" t="str"/>
+      <x:c r="O26" s="33" t="str"/>
+      <x:c r="P26" s="33" t="str"/>
+      <x:c r="Q26" s="36" t="str"/>
+      <x:c r="R26" s="51" t="str"/>
+      <x:c r="S26" s="36" t="str"/>
       <x:c r="T26" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -9302,41 +8818,19 @@
       <x:c r="H27" s="36" t="str">
         <x:v>https://inetl-ip.gov.tl/</x:v>
       </x:c>
-      <x:c r="I27" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J27" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K27" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L27" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M27" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N27" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O27" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P27" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q27" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R27" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S27" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/TLS/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I27" s="33" t="str"/>
+      <x:c r="J27" s="36" t="str"/>
+      <x:c r="K27" s="36" t="str"/>
+      <x:c r="L27" s="36" t="str"/>
+      <x:c r="M27" s="33" t="str"/>
+      <x:c r="N27" s="48" t="str"/>
+      <x:c r="O27" s="33" t="str"/>
+      <x:c r="P27" s="33" t="str"/>
+      <x:c r="Q27" s="36" t="str"/>
+      <x:c r="R27" s="51" t="str"/>
+      <x:c r="S27" s="36" t="str"/>
       <x:c r="T27" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -9360,41 +8854,19 @@
       <x:c r="H28" s="36" t="str">
         <x:v>https://stat.gov.tm/en/</x:v>
       </x:c>
-      <x:c r="I28" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J28" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K28" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L28" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M28" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N28" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O28" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P28" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q28" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R28" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S28" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/TKM/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I28" s="33" t="str"/>
+      <x:c r="J28" s="36" t="str"/>
+      <x:c r="K28" s="36" t="str"/>
+      <x:c r="L28" s="36" t="str"/>
+      <x:c r="M28" s="33" t="str"/>
+      <x:c r="N28" s="48" t="str"/>
+      <x:c r="O28" s="33" t="str"/>
+      <x:c r="P28" s="33" t="str"/>
+      <x:c r="Q28" s="36" t="str"/>
+      <x:c r="R28" s="51" t="str"/>
+      <x:c r="S28" s="36" t="str"/>
       <x:c r="T28" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -9422,41 +8894,19 @@
       <x:c r="H29" s="36" t="str">
         <x:v>https://www.ubos.org/?p_id=104&amp;pagename=explore-publications</x:v>
       </x:c>
-      <x:c r="I29" s="33" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="J29" s="36" t="str">
-        <x:v>gdp_deflator</x:v>
-      </x:c>
-      <x:c r="K29" s="36" t="str">
-        <x:v>GDP deflator (base year varies by country)</x:v>
-      </x:c>
-      <x:c r="L29" s="36" t="str">
-        <x:v>World Bank, World Development Indicators</x:v>
-      </x:c>
-      <x:c r="M29" s="33" t="str">
-        <x:v>annual</x:v>
-      </x:c>
-      <x:c r="N29" s="48" t="str">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="O29" s="33" t="str">
-        <x:v>2015</x:v>
-      </x:c>
-      <x:c r="P29" s="33" t="str">
-        <x:v>2025</x:v>
-      </x:c>
-      <x:c r="Q29" s="36" t="str">
-        <x:v>published</x:v>
-      </x:c>
-      <x:c r="R29" s="51" t="n">
-        <x:v>46232.95527777778</x:v>
-      </x:c>
-      <x:c r="S29" s="36" t="str">
-        <x:v>https://api.worldbank.org/v2/country/UGA/indicator/NY.GDP.DEFL.ZS</x:v>
-      </x:c>
+      <x:c r="I29" s="33" t="str"/>
+      <x:c r="J29" s="36" t="str"/>
+      <x:c r="K29" s="36" t="str"/>
+      <x:c r="L29" s="36" t="str"/>
+      <x:c r="M29" s="33" t="str"/>
+      <x:c r="N29" s="48" t="str"/>
+      <x:c r="O29" s="33" t="str"/>
+      <x:c r="P29" s="33" t="str"/>
+      <x:c r="Q29" s="36" t="str"/>
+      <x:c r="R29" s="51" t="str"/>
+      <x:c r="S29" s="36" t="str"/>
       <x:c r="T29" s="36" t="str">
-        <x:v>상위지수 미적재 또는 기간 미충족 시 거시지표 대체; 보고서에 한계 명시</x:v>
+        <x:v>국가 공식 실제 시계열 미적재; 자동보정 불가</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -9530,7 +8980,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2e3ebfb67d1446a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a0f60ed1ca1440a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9631,7 +9081,7 @@
         <x:v>evidence</x:v>
       </x:c>
       <x:c r="B9" s="36" t="str">
-        <x:v>자동 추출 수치근거 3,563건</x:v>
+        <x:v>자동 추출 수치근거 4,402건</x:v>
       </x:c>
       <x:c r="C9" s="36" t="str">
         <x:v>evidence_id, bid_no</x:v>
@@ -9742,7 +9192,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa82d875f97b415c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf027fa4ee53c4081"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9830,7 +9280,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd33f14f98d84534"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60aff41fa3d44132"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>